<commit_message>
Fix sensor ID parsing, eliminate postmile float artifacts, and apply bare-bones serif styling
</commit_message>
<xml_diff>
--- a/staging/Master_CA_Project_List_Cleaned.xlsx
+++ b/staging/Master_CA_Project_List_Cleaned.xlsx
@@ -2970,7 +2970,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>146.19999999999999</t>
+          <t>146.2</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>146.19999999999999</t>
+          <t>146.2</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -3695,7 +3695,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>38.299999999999997</t>
+          <t>38.3</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>139.80000000000001</t>
+          <t>139.8</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -4068,12 +4068,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>R18.100</t>
+          <t>R18.1</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>20.100000000000001</t>
+          <t>20.1</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>66.278999999999996</t>
+          <t>66.279</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -4930,7 +4930,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>8.8000000000000007</t>
+          <t>8.8</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -5344,7 +5344,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>8.8000000000000007</t>
+          <t>8.8</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -5749,7 +5749,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>38.700000000000003</t>
+          <t>38.7</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -6146,7 +6146,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>9.3000000000000007</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -6786,7 +6786,7 @@
       <c r="BL16" t="inlineStr"/>
       <c r="BM16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN16" t="inlineStr">
@@ -7264,7 +7264,7 @@
       <c r="BL17" t="inlineStr"/>
       <c r="BM17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN17" t="inlineStr">
@@ -9054,7 +9054,7 @@
       </c>
       <c r="BM21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN21" t="inlineStr">
@@ -9099,7 +9099,7 @@
       </c>
       <c r="BV21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BW21" t="inlineStr">
@@ -9444,7 +9444,7 @@
       </c>
       <c r="BM22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN22" t="inlineStr">
@@ -9846,7 +9846,7 @@
       </c>
       <c r="BM23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN23" t="inlineStr">
@@ -10085,7 +10085,7 @@
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA24" t="inlineStr">
@@ -10359,7 +10359,7 @@
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA25" t="inlineStr">
@@ -10828,7 +10828,7 @@
       </c>
       <c r="BM26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN26" t="inlineStr">
@@ -11254,7 +11254,7 @@
       </c>
       <c r="BM27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN27" t="inlineStr">
@@ -11458,7 +11458,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>12.234999999999999</t>
+          <t>12.235</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -11713,7 +11713,7 @@
       </c>
       <c r="BM28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN28" t="inlineStr">
@@ -11965,7 +11965,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>40.299999999999997</t>
+          <t>40.3</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -12020,7 +12020,7 @@
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="AA29" t="inlineStr">
@@ -12211,7 +12211,7 @@
       <c r="BL29" t="inlineStr"/>
       <c r="BM29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN29" t="inlineStr">
@@ -12466,7 +12466,7 @@
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="AA30" t="inlineStr">
@@ -12657,7 +12657,7 @@
       <c r="BL30" t="inlineStr"/>
       <c r="BM30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN30" t="inlineStr">
@@ -13075,7 +13075,7 @@
       <c r="BL31" t="inlineStr"/>
       <c r="BM31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN31" t="inlineStr">
@@ -13116,7 +13116,7 @@
       <c r="BU31" t="inlineStr"/>
       <c r="BV31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BW31" t="inlineStr">
@@ -13549,7 +13549,7 @@
       <c r="BL32" t="inlineStr"/>
       <c r="BM32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN32" t="inlineStr">
@@ -13672,7 +13672,7 @@
       <c r="CM32" t="inlineStr"/>
       <c r="CN32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="CO32" t="inlineStr">
@@ -13785,12 +13785,12 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>34.299999999999997</t>
+          <t>34.3</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>34.700000000000003</t>
+          <t>34.7</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -14047,7 +14047,7 @@
       <c r="BL33" t="inlineStr"/>
       <c r="BM33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN33" t="inlineStr">
@@ -14188,7 +14188,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>72.900000000000006</t>
+          <t>72.9</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -14203,7 +14203,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>323.39999999999998</t>
+          <t>323.4</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -14895,7 +14895,7 @@
       <c r="BL35" t="inlineStr"/>
       <c r="BM35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN35" t="inlineStr">
@@ -15293,7 +15293,7 @@
       <c r="BL36" t="inlineStr"/>
       <c r="BM36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN36" t="inlineStr">
@@ -15695,7 +15695,7 @@
       <c r="BL37" t="inlineStr"/>
       <c r="BM37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN37" t="inlineStr">
@@ -16141,7 +16141,7 @@
       <c r="BL38" t="inlineStr"/>
       <c r="BM38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN38" t="inlineStr">
@@ -16365,7 +16365,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>R7.500</t>
+          <t>R7.5</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -16631,7 +16631,7 @@
       <c r="BL39" t="inlineStr"/>
       <c r="BM39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN39" t="inlineStr">
@@ -16847,7 +16847,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>R7.500</t>
+          <t>R7.5</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -17113,7 +17113,7 @@
       <c r="BL40" t="inlineStr"/>
       <c r="BM40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN40" t="inlineStr">
@@ -18098,7 +18098,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>33.200000000000003</t>
+          <t>33.2</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -18484,7 +18484,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>33.200000000000003</t>
+          <t>33.2</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -19895,7 +19895,7 @@
       <c r="BL47" t="inlineStr"/>
       <c r="BM47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN47" t="inlineStr">
@@ -20337,7 +20337,7 @@
       <c r="BL48" t="inlineStr"/>
       <c r="BM48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN48" t="inlineStr">
@@ -21018,7 +21018,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>143.30000000000001</t>
+          <t>143.3</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -21249,7 +21249,7 @@
       <c r="BL50" t="inlineStr"/>
       <c r="BM50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN50" t="inlineStr">
@@ -21440,7 +21440,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>143.30000000000001</t>
+          <t>143.3</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -21671,7 +21671,7 @@
       <c r="BL51" t="inlineStr"/>
       <c r="BM51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN51" t="inlineStr">
@@ -21871,7 +21871,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>40.200000000000003</t>
+          <t>40.2</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -22117,7 +22117,7 @@
       </c>
       <c r="BM52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN52" t="inlineStr">
@@ -22329,7 +22329,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>40.200000000000003</t>
+          <t>40.2</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -22575,7 +22575,7 @@
       </c>
       <c r="BM53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN53" t="inlineStr">
@@ -22974,11 +22974,7 @@
       <c r="BY54" t="inlineStr"/>
       <c r="BZ54" t="inlineStr"/>
       <c r="CA54" t="inlineStr"/>
-      <c r="CB54" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
+      <c r="CB54" t="inlineStr"/>
       <c r="CC54" t="inlineStr"/>
       <c r="CD54" t="inlineStr"/>
       <c r="CE54" t="inlineStr"/>
@@ -22986,11 +22982,7 @@
       <c r="CG54" t="inlineStr"/>
       <c r="CH54" t="inlineStr"/>
       <c r="CI54" t="inlineStr"/>
-      <c r="CJ54" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
+      <c r="CJ54" t="inlineStr"/>
       <c r="CK54" t="inlineStr"/>
       <c r="CL54" t="inlineStr"/>
       <c r="CM54" t="inlineStr"/>
@@ -23106,7 +23098,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>I-10 30.3</t>
+          <t>30.3</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -23553,7 +23545,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>I-10 30.3</t>
+          <t>30.3</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -24257,7 +24249,7 @@
       <c r="BL57" t="inlineStr"/>
       <c r="BM57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN57" t="inlineStr">
@@ -24332,7 +24324,7 @@
       <c r="CM57" t="inlineStr"/>
       <c r="CN57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="CO57" t="inlineStr">
@@ -24707,7 +24699,7 @@
       <c r="BL58" t="inlineStr"/>
       <c r="BM58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN58" t="inlineStr">
@@ -25137,7 +25129,7 @@
       <c r="BL59" t="inlineStr"/>
       <c r="BM59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN59" t="inlineStr">
@@ -25563,7 +25555,7 @@
       <c r="BL60" t="inlineStr"/>
       <c r="BM60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN60" t="inlineStr">
@@ -25993,7 +25985,7 @@
       <c r="BL61" t="inlineStr"/>
       <c r="BM61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN61" t="inlineStr">
@@ -26383,7 +26375,7 @@
       <c r="BL62" t="inlineStr"/>
       <c r="BM62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN62" t="inlineStr">
@@ -26747,11 +26739,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="BI63" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
+      <c r="BI63" t="inlineStr"/>
       <c r="BJ63" t="inlineStr"/>
       <c r="BK63" t="inlineStr"/>
       <c r="BL63" t="inlineStr"/>
@@ -26760,16 +26748,8 @@
       <c r="BO63" t="inlineStr"/>
       <c r="BP63" t="inlineStr"/>
       <c r="BQ63" t="inlineStr"/>
-      <c r="BR63" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="BS63" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
+      <c r="BR63" t="inlineStr"/>
+      <c r="BS63" t="inlineStr"/>
       <c r="BT63" t="inlineStr"/>
       <c r="BU63" t="inlineStr"/>
       <c r="BV63" t="inlineStr"/>
@@ -26777,16 +26757,8 @@
       <c r="BX63" t="inlineStr"/>
       <c r="BY63" t="inlineStr"/>
       <c r="BZ63" t="inlineStr"/>
-      <c r="CA63" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="CB63" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
+      <c r="CA63" t="inlineStr"/>
+      <c r="CB63" t="inlineStr"/>
       <c r="CC63" t="inlineStr"/>
       <c r="CD63" t="inlineStr"/>
       <c r="CE63" t="inlineStr"/>
@@ -26794,11 +26766,7 @@
       <c r="CG63" t="inlineStr"/>
       <c r="CH63" t="inlineStr"/>
       <c r="CI63" t="inlineStr"/>
-      <c r="CJ63" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
+      <c r="CJ63" t="inlineStr"/>
       <c r="CK63" t="inlineStr"/>
       <c r="CL63" t="inlineStr"/>
       <c r="CM63" t="inlineStr"/>
@@ -27179,7 +27147,7 @@
       <c r="BL64" t="inlineStr"/>
       <c r="BM64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN64" t="inlineStr">
@@ -27254,7 +27222,7 @@
       <c r="CM64" t="inlineStr"/>
       <c r="CN64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="CO64" t="inlineStr">
@@ -27629,7 +27597,7 @@
       <c r="BL65" t="inlineStr"/>
       <c r="BM65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN65" t="inlineStr">
@@ -27704,7 +27672,7 @@
       <c r="CM65" t="inlineStr"/>
       <c r="CN65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="CO65" t="inlineStr">
@@ -27837,7 +27805,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>148.19999999999999</t>
+          <t>148.2</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -28251,7 +28219,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>148.19999999999999</t>
+          <t>148.2</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -28641,7 +28609,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>37.200000000000003</t>
+          <t>37.2</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
@@ -28656,7 +28624,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>35.700000000000003</t>
+          <t>35.7</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -28907,7 +28875,7 @@
       <c r="BL68" t="inlineStr"/>
       <c r="BM68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN68" t="inlineStr">
@@ -29079,7 +29047,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>37.200000000000003</t>
+          <t>37.2</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
@@ -29094,7 +29062,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>35.700000000000003</t>
+          <t>35.7</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -29345,7 +29313,7 @@
       <c r="BL69" t="inlineStr"/>
       <c r="BM69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN69" t="inlineStr">
@@ -31801,7 +31769,7 @@
       </c>
       <c r="BM75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN75" t="inlineStr">
@@ -32748,7 +32716,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>65.400000000000006</t>
+          <t>65.4</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -32979,11 +32947,7 @@
       <c r="BY78" t="inlineStr"/>
       <c r="BZ78" t="inlineStr"/>
       <c r="CA78" t="inlineStr"/>
-      <c r="CB78" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
+      <c r="CB78" t="inlineStr"/>
       <c r="CC78" t="inlineStr"/>
       <c r="CD78" t="inlineStr"/>
       <c r="CE78" t="inlineStr"/>
@@ -32991,11 +32955,7 @@
       <c r="CG78" t="inlineStr"/>
       <c r="CH78" t="inlineStr"/>
       <c r="CI78" t="inlineStr"/>
-      <c r="CJ78" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
+      <c r="CJ78" t="inlineStr"/>
       <c r="CK78" t="inlineStr"/>
       <c r="CL78" t="inlineStr"/>
       <c r="CM78" t="inlineStr"/>
@@ -33130,7 +33090,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>19.600000000000001</t>
+          <t>19.6</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
@@ -33508,7 +33468,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>19.600000000000001</t>
+          <t>19.6</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -33881,7 +33841,7 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>9.3000000000000007</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
@@ -35517,7 +35477,7 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>71.400000000000006</t>
+          <t>71.4</t>
         </is>
       </c>
       <c r="O85" t="inlineStr">
@@ -35919,7 +35879,7 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>71.400000000000006</t>
+          <t>71.4</t>
         </is>
       </c>
       <c r="O86" t="inlineStr">
@@ -37385,7 +37345,7 @@
       </c>
       <c r="BV89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BW89" t="inlineStr">
@@ -37843,7 +37803,7 @@
       </c>
       <c r="BV90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BW90" t="inlineStr">
@@ -39033,7 +38993,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>16.600000000000001</t>
+          <t>16.6</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
@@ -39395,7 +39355,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>16.600000000000001</t>
+          <t>16.6</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
@@ -39763,7 +39723,7 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>149.80000000000001</t>
+          <t>149.8</t>
         </is>
       </c>
       <c r="O95" t="inlineStr">
@@ -40177,7 +40137,7 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>149.80000000000001</t>
+          <t>149.8</t>
         </is>
       </c>
       <c r="O96" t="inlineStr">
@@ -40591,12 +40551,12 @@
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>77.921000000000006</t>
+          <t>77.921</t>
         </is>
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>77.921000000000006</t>
+          <t>77.921</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
@@ -42046,7 +42006,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>37.299999999999997</t>
+          <t>37.3</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
@@ -42308,7 +42268,7 @@
       <c r="BL101" t="inlineStr"/>
       <c r="BM101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN101" t="inlineStr">
@@ -42537,7 +42497,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>37.299999999999997</t>
+          <t>37.3</t>
         </is>
       </c>
       <c r="M102" t="inlineStr">
@@ -42799,7 +42759,7 @@
       <c r="BL102" t="inlineStr"/>
       <c r="BM102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN102" t="inlineStr">
@@ -44437,7 +44397,7 @@
       <c r="BL106" t="inlineStr"/>
       <c r="BM106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN106" t="inlineStr">
@@ -44815,7 +44775,7 @@
       <c r="BL107" t="inlineStr"/>
       <c r="BM107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN107" t="inlineStr">
@@ -44960,7 +44920,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>39.799999999999997</t>
+          <t>39.8</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">
@@ -44970,12 +44930,12 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>37.299999999999997</t>
+          <t>37.3</t>
         </is>
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>39.700000000000003</t>
+          <t>39.7</t>
         </is>
       </c>
       <c r="P108" t="inlineStr">
@@ -45221,7 +45181,7 @@
       <c r="BL108" t="inlineStr"/>
       <c r="BM108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN108" t="inlineStr">
@@ -45378,7 +45338,7 @@
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>39.799999999999997</t>
+          <t>39.8</t>
         </is>
       </c>
       <c r="M109" t="inlineStr">
@@ -45388,12 +45348,12 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>37.299999999999997</t>
+          <t>37.3</t>
         </is>
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>39.700000000000003</t>
+          <t>39.7</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
@@ -45639,7 +45599,7 @@
       <c r="BL109" t="inlineStr"/>
       <c r="BM109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mainlane </t>
+          <t>Mainlane</t>
         </is>
       </c>
       <c r="BN109" t="inlineStr">
@@ -45812,7 +45772,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>1.1000000000000001</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="M110" t="inlineStr">
@@ -45827,7 +45787,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2.9590000000000001</t>
+          <t>2.959</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
@@ -45850,11 +45810,7 @@
           <t>suburban</t>
         </is>
       </c>
-      <c r="T110" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="T110" t="inlineStr"/>
       <c r="U110" t="inlineStr"/>
       <c r="V110" t="inlineStr">
         <is>
@@ -45864,11 +45820,7 @@
       <c r="W110" t="inlineStr"/>
       <c r="X110" t="inlineStr"/>
       <c r="Y110" t="inlineStr"/>
-      <c r="Z110" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="Z110" t="inlineStr"/>
       <c r="AA110" t="inlineStr"/>
       <c r="AB110" t="inlineStr">
         <is>
@@ -46164,12 +46116,12 @@
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>7.2119999999999997</t>
+          <t>7.212</t>
         </is>
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>7.2119999999999997</t>
+          <t>7.212</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
@@ -46194,7 +46146,7 @@
       </c>
       <c r="T111" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="U111" t="inlineStr">
@@ -46212,7 +46164,7 @@
       <c r="Y111" t="inlineStr"/>
       <c r="Z111" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA111" t="inlineStr">
@@ -46534,12 +46486,12 @@
       </c>
       <c r="N112" t="inlineStr">
         <is>
-          <t>6.7009999999999996</t>
+          <t>6.701</t>
         </is>
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>8.4860000000000007</t>
+          <t>8.486</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
@@ -46564,7 +46516,7 @@
       </c>
       <c r="T112" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="U112" t="inlineStr">
@@ -46594,7 +46546,7 @@
       </c>
       <c r="Z112" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="AA112" t="inlineStr">
@@ -47018,37 +46970,37 @@
       </c>
       <c r="T113" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="W113" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y113" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z113" t="inlineStr">
+        <is>
           <t>6</t>
-        </is>
-      </c>
-      <c r="U113" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="V113" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="W113" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X113" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Y113" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Z113" t="inlineStr">
-        <is>
-          <t>8</t>
         </is>
       </c>
       <c r="AA113" t="inlineStr">
@@ -47376,7 +47328,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>34.200000000000003</t>
+          <t>34.2</t>
         </is>
       </c>
       <c r="M114" t="inlineStr">
@@ -47870,7 +47822,7 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>34.200000000000003</t>
+          <t>34.2</t>
         </is>
       </c>
       <c r="M115" t="inlineStr">
@@ -48395,7 +48347,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>75.900000000000006</t>
+          <t>75.9</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -48841,7 +48793,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>75.900000000000006</t>
+          <t>75.9</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -49268,7 +49220,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>8.6999999999999993</t>
+          <t>8.7</t>
         </is>
       </c>
       <c r="M118" t="inlineStr">
@@ -49278,12 +49230,12 @@
       </c>
       <c r="N118" t="inlineStr">
         <is>
-          <t>78.400000000000006</t>
+          <t>78.4</t>
         </is>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>80.900000000000006</t>
+          <t>80.9</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -49547,7 +49499,7 @@
       <c r="BR118" t="inlineStr"/>
       <c r="BS118" t="inlineStr">
         <is>
-          <t xml:space="preserve">1204395+1210063 (HOV)	</t>
+          <t>1204395+1210063 (HOV)</t>
         </is>
       </c>
       <c r="BT118" t="inlineStr">
@@ -49702,7 +49654,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>8.6999999999999993</t>
+          <t>8.7</t>
         </is>
       </c>
       <c r="M119" t="inlineStr">
@@ -49712,12 +49664,12 @@
       </c>
       <c r="N119" t="inlineStr">
         <is>
-          <t>78.400000000000006</t>
+          <t>78.4</t>
         </is>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>80.900000000000006</t>
+          <t>80.9</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">

</xml_diff>

<commit_message>
Publish preparation: refactor core engine, add PeMS batch downloader, and update docs
</commit_message>
<xml_diff>
--- a/staging/Master_CA_Project_List_Cleaned.xlsx
+++ b/staging/Master_CA_Project_List_Cleaned.xlsx
@@ -10359,12 +10359,12 @@
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>1(for 2 miles)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AD25" t="inlineStr">
@@ -12020,7 +12020,7 @@
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="AA29" t="inlineStr">
@@ -12466,7 +12466,7 @@
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="AA30" t="inlineStr">
@@ -45810,7 +45810,11 @@
           <t>suburban</t>
         </is>
       </c>
-      <c r="T110" t="inlineStr"/>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="U110" t="inlineStr"/>
       <c r="V110" t="inlineStr">
         <is>
@@ -45820,7 +45824,11 @@
       <c r="W110" t="inlineStr"/>
       <c r="X110" t="inlineStr"/>
       <c r="Y110" t="inlineStr"/>
-      <c r="Z110" t="inlineStr"/>
+      <c r="Z110" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="AA110" t="inlineStr"/>
       <c r="AB110" t="inlineStr">
         <is>
@@ -46146,7 +46154,7 @@
       </c>
       <c r="T111" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="U111" t="inlineStr">
@@ -46164,7 +46172,7 @@
       <c r="Y111" t="inlineStr"/>
       <c r="Z111" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA111" t="inlineStr">
@@ -46516,37 +46524,37 @@
       </c>
       <c r="T112" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V112" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W112" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X112" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y112" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z112" t="inlineStr">
+        <is>
           <t>8</t>
-        </is>
-      </c>
-      <c r="U112" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="V112" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="W112" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X112" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Y112" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Z112" t="inlineStr">
-        <is>
-          <t>10</t>
         </is>
       </c>
       <c r="AA112" t="inlineStr">
@@ -46970,7 +46978,7 @@
       </c>
       <c r="T113" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="U113" t="inlineStr">
@@ -47000,7 +47008,7 @@
       </c>
       <c r="Z113" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA113" t="inlineStr">

</xml_diff>